<commit_message>
Improved update system with smart input handling
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4212" yWindow="3360" windowWidth="17280" windowHeight="8880" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,11 +16,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
@@ -45,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -424,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -504,49 +512,51 @@
           <t>01-06-2026</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Rahul Kumar</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Ramesh Kumar</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>Sita Devi</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>Chennai</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9876543210</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>ABC Public School</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
         <is>
           <t>New Admission</t>
         </is>
       </c>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="n">

</xml_diff>

<commit_message>
Added README and cleaned repository structure
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -547,12 +547,12 @@
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="K2" s="1" t="inlineStr">
         <is>
-          <t>New Admission</t>
+          <t>LEFT STUDENT | Reason: schooling done | Remarks: good</t>
         </is>
       </c>
       <c r="L2" s="1" t="n"/>

</xml_diff>

<commit_message>
feat: add Flask web frontend with full UI (dashboard, search, admission, edit, leave)
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1300,6 +1300,57 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>kumar karthikk</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>uma maheswara rao</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>lakshmi</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>srikakulam</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>7207256386</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>xyz</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>